<commit_message>
Add footer to DQA template and required attribution licensing
</commit_message>
<xml_diff>
--- a/docs/04-architecture-design/DataQualityAssessment.xlsx
+++ b/docs/04-architecture-design/DataQualityAssessment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\git\ai-ml-engineering-framework\docs\04-architecture-design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA7CC19-9BFB-4B12-819A-1E6F3378CA52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47489E18-32DD-4A26-8EF7-5ED49225597D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test List" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="62">
   <si>
     <t>DQA ID</t>
   </si>
@@ -204,13 +204,19 @@
   </si>
   <si>
     <t>Automated profiling with configurable missing-value sentinels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/iainjclark/ai-ml-engineering-framework </t>
+  </si>
+  <si>
+    <t>Generated using the AI/ML Engineering Framework — Iain J. Clark, PhD. Attribution required; see NOTICE.md.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -257,6 +263,20 @@
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Georgia"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF444444"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -307,10 +327,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -337,6 +358,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -344,11 +367,19 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF444444"/>
+      <color rgb="FF999999"/>
+      <color rgb="FF666666"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -698,7 +729,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:J12"/>
+  <dimension ref="B2:J15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
@@ -712,17 +743,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
@@ -806,6 +837,16 @@
       <c r="H12" s="6"/>
       <c r="I12" s="2"/>
       <c r="J12" s="6"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C15" s="10" t="s">
+        <v>60</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -813,11 +854,12 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B12" location="'C01'!A1" display="C01" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C15" r:id="rId1" xr:uid="{39AE6939-611F-4386-84DC-F218C1ECEC11}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -827,7 +869,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:X21"/>
+  <dimension ref="B2:X24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.7109375" customWidth="1"/>
@@ -851,58 +893,58 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10"/>
-      <c r="S2" s="10"/>
-      <c r="T2" s="10"/>
-      <c r="U2" s="10"/>
-      <c r="V2" s="10"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
-      <c r="S3" s="11"/>
-      <c r="T3" s="11"/>
-      <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
-      <c r="W3" s="11"/>
-      <c r="X3" s="11"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
+      <c r="V3" s="13"/>
+      <c r="W3" s="13"/>
+      <c r="X3" s="13"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
@@ -1175,15 +1217,28 @@
       <c r="W21" s="6"/>
       <c r="X21" s="2"/>
     </row>
+    <row r="23" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="C23" s="11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="C24" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:X2"/>
     <mergeCell ref="B3:X3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C24" r:id="rId1" xr:uid="{962E391A-A7F7-4634-9AEC-ADC6C7C2B230}"/>
+  </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>